<commit_message>
stage 1 stage 2 followup done
</commit_message>
<xml_diff>
--- a/forms/contact/participant-create.xlsx
+++ b/forms/contact/participant-create.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,13 +27,28 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003A5234"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -48,8 +63,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,493 +434,684 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>hint</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>appearance</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>relevant</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>calculation</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>constraint</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>constraint_message</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>default</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>inputs</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>false()</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>user</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>contact_id</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>facility_id</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>participant</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>PARENT</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>participant</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Full Name</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>age</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Age</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= 130</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Age must be between 0 and 130</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>select_one gender_list</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Gender</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>tel</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Phone Number</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>true()</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>Please enter a valid phone number.</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>select_one education_list</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>education_level</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Education level</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Used to select the correct HMSE cut-off in Stage 2.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>informant_name</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Family member / informant name</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>The person who can answer the AD8 in Stage 2.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>tel</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>informant_phone</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Informant phone number</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>true()</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Please enter a valid phone number.</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>select_one yes_no</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>consent_given</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Consent given for screening and data storage?</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Explain purpose, confidentiality and the right to stop at any time before recording this.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>consent_recorded_at</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>consent_version</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>'SATORU-CONSENT-v1.0-2026'</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>multiline</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -914,74 +1124,147 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>list_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>gender_list</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>male</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>gender_list</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>female</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>gender_list</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Other</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>education_list</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>illiterate</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>No formal schooling / cannot read</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>education_list</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>primary</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>1-7 years of schooling</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>education_list</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>secondary_plus</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>8 years or more</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>yes_no</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>yes_no</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -998,46 +1281,52 @@
   </sheetPr>
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>form_title</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>form_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>version</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>default_language</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>New Participant</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>contact:participant:create</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-07-27 00-00</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-29 00-00</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>en</t>
         </is>

</xml_diff>

<commit_message>
updated patient registration form and added the asessment form and cr no logic
</commit_message>
<xml_diff>
--- a/forms/contact/participant-create.xlsx
+++ b/forms/contact/participant-create.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,27 +28,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="003A5234"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -63,12 +51,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,21 +419,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -508,610 +480,589 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>inputs</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>field-list</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>false()</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>user</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>contact_id</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>facility_id</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>begin group</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>participant</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Participant</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>hidden</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>parent</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>PARENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>hidden</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>parent</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>NO_LABEL</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>PARENT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>hidden</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>NO_LABEL</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>participant</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Full Name</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>cr_no</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CR (Case Record) No.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Check for an existing participant with this CR No. before creating a new one to avoid duplicates.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>aadhaar_last4</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Aadhaar (last 4 digits)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>age</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Age</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>. &gt;= 0 and . &lt;= 130</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Age must be between 0 and 130</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>select_one gender_list</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Gender</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>select_one education_list</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>education_level</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Education level</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Used to select the correct HMSE cut-off in Stage 2.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>occupation</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Occupation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>tel</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Phone Number</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Phone (patient / caregiver / attendant)</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>true()</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>Please enter a valid phone number.</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>select_one education_list</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>education_level</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Education level</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Used to select the correct HMSE cut-off in Stage 2.</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>address</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Address / Locality</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>referral_department</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Department (referral)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>referred_by</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Referred by (doctor name)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>referral_complaint</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Health complaint &amp; reason for referral</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>informant_name</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Respondent name &amp; relation</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>tel</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>informant_phone</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Informant phone number</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>true()</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Please enter a valid phone number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>select_one consent_mode_list</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>consent_mode</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Type of consent obtained</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>select_one yes_no</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>consent_given</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Consent given for screening and data storage?</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Explain purpose, confidentiality and the right to stop at any time before recording this.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>consent_recorded_at</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>consent_version</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>'SATORU-CONSENT-v1.0-2026'</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>informant_name</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Family member / informant name</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>The person who can answer the AD8 in Stage 2.</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>tel</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>informant_phone</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Informant phone number</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>true()</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>Please enter a valid phone number.</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>select_one yes_no</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>consent_given</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Consent given for screening and data storage?</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Explain purpose, confidentiality and the right to stop at any time before recording this.</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>consent_recorded_at</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>calculate</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>consent_version</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>'SATORU-CONSENT-v1.0-2026'</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>multiline</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr"/>
-      <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1124,13 +1075,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1150,119 +1096,153 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>gender_list</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>male</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>gender_list</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>female</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>education_list</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>illiterate</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>No formal schooling / cannot read</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>education_list</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>1-7 years of schooling</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>education_list</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>secondary_plus</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>8 years or more</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>consent_mode_list</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>written</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Written</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>consent_mode_list</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>verbal</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Verbal</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>yes_no</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>yes_no</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1281,12 +1261,6 @@
   </sheetPr>
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1311,22 +1285,22 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>New Participant</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>contact:participant:create</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-29 00-00</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-08-12 00-00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>en</t>
         </is>

</xml_diff>